<commit_message>
Update prices from Google Sheets
</commit_message>
<xml_diff>
--- a/public/projects.xlsx
+++ b/public/projects.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="89">
   <si>
     <t>Project</t>
   </si>
@@ -3239,6 +3239,9 @@
       </c>
     </row>
     <row r="51">
+      <c r="A51" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="E51" s="3" t="s">
         <v>54</v>
       </c>

</xml_diff>